<commit_message>
#2 Fresh Deliverables generated.
</commit_message>
<xml_diff>
--- a/Design-Files/DBS-Stepper-Module/BOM/Altium_BOM-Latest-v1.0.xlsx
+++ b/Design-Files/DBS-Stepper-Module/BOM/Altium_BOM-Latest-v1.0.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="502" uniqueCount="332">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="502" uniqueCount="333">
   <si>
     <t>Description</t>
   </si>
@@ -1023,6 +1023,9 @@
   </si>
   <si>
     <t>Aliexpress</t>
+  </si>
+  <si>
+    <t>VSSOP-8</t>
   </si>
 </sst>
 </file>
@@ -1495,9 +1498,9 @@
   <cols>
     <col min="1" max="1" width="9.140625" style="6"/>
     <col min="2" max="2" width="13" style="6" customWidth="1"/>
-    <col min="3" max="4" width="23.140625" style="6" customWidth="1"/>
-    <col min="5" max="5" width="19.7109375" style="6" hidden="1" customWidth="1"/>
-    <col min="6" max="7" width="16.5703125" style="6" customWidth="1"/>
+    <col min="3" max="3" width="23.140625" style="6" customWidth="1"/>
+    <col min="4" max="6" width="41.5703125" style="6" customWidth="1"/>
+    <col min="7" max="7" width="16.5703125" style="6" customWidth="1"/>
     <col min="8" max="8" width="17.7109375" style="6" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="12" style="6" customWidth="1"/>
     <col min="10" max="10" width="22.85546875" bestFit="1" customWidth="1"/>
@@ -3583,7 +3586,7 @@
       <c r="J67" s="1"/>
       <c r="K67" s="1"/>
     </row>
-    <row r="68" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A68" s="4">
         <v>67</v>
       </c>
@@ -3631,7 +3634,7 @@
         <v>296</v>
       </c>
       <c r="E69" s="5" t="s">
-        <v>295</v>
+        <v>332</v>
       </c>
       <c r="F69" s="5" t="s">
         <v>295</v>

</xml_diff>